<commit_message>
new data reduction results
</commit_message>
<xml_diff>
--- a/Results/data_reduction_results/diagnostics/pam_parametrizer_diagnostics_datareduc_70_1.xlsx
+++ b/Results/data_reduction_results/diagnostics/pam_parametrizer_diagnostics_datareduc_70_1.xlsx
@@ -80485,7 +80485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80505,7 +80505,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.04579747052962768</v>
+        <v>0.3360869971578732</v>
       </c>
     </row>
     <row r="3">
@@ -80513,7 +80513,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04579747051893731</v>
+        <v>0.3360869971581927</v>
       </c>
     </row>
     <row r="4">
@@ -80521,7 +80521,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.04579746351818592</v>
+        <v>0.3360869971578467</v>
       </c>
     </row>
     <row r="5">
@@ -80529,7 +80529,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.04579745442420143</v>
+        <v>0.3360869971580439</v>
       </c>
     </row>
     <row r="6">
@@ -80537,6 +80537,646 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
+        <v>0.3360869971577342</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-0.09799184133140681</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-0.09799184133170566</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-0.09799184132387981</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-0.09799184133579578</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.09799184133578348</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2136717049355444</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.2135951910399787</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.2137265044921353</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2139829785673774</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.2140358226517614</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-5.871800401103894</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" t="n">
+        <v>-5.871800401103775</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" t="n">
+        <v>-5.871800401103808</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" t="n">
+        <v>-5.871800401103748</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>5</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-5.871800401103648</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" t="n">
+        <v>-1.77372981173008</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" t="n">
+        <v>-1.761280235997502</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" t="n">
+        <v>-1.759859242566967</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" t="n">
+        <v>-1.755705941697224</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" t="n">
+        <v>-1.729010014722867</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" t="n">
+        <v>0.3458127812505523</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" t="n">
+        <v>0.3490016206945754</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0.348863131071253</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>4</v>
+      </c>
+      <c r="B30" t="n">
+        <v>0.394738225243877</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" t="n">
+        <v>0.3959558733673551</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" t="n">
+        <v>0.2023554802528108</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" t="n">
+        <v>0.2022602424175468</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>3</v>
+      </c>
+      <c r="B34" t="n">
+        <v>0.2021896114763853</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>4</v>
+      </c>
+      <c r="B35" t="n">
+        <v>0.2924465481806777</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>5</v>
+      </c>
+      <c r="B36" t="n">
+        <v>0.3835147883380022</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>1</v>
+      </c>
+      <c r="B37" t="n">
+        <v>0.6182408586372247</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" t="n">
+        <v>0.6183161048256467</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>3</v>
+      </c>
+      <c r="B39" t="n">
+        <v>0.6183277772609176</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>4</v>
+      </c>
+      <c r="B40" t="n">
+        <v>0.6183277772989128</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>5</v>
+      </c>
+      <c r="B41" t="n">
+        <v>0.6183361253775708</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>1</v>
+      </c>
+      <c r="B42" t="n">
+        <v>-1.190236601262407</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" t="n">
+        <v>-1.19023660126345</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>3</v>
+      </c>
+      <c r="B44" t="n">
+        <v>-1.19023660125767</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>4</v>
+      </c>
+      <c r="B45" t="n">
+        <v>-1.190236601138187</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>5</v>
+      </c>
+      <c r="B46" t="n">
+        <v>-1.19023660125568</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" t="n">
+        <v>-1.71450287112016</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" t="n">
+        <v>-1.714502871339683</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>3</v>
+      </c>
+      <c r="B49" t="n">
+        <v>-1.714502871111872</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>4</v>
+      </c>
+      <c r="B50" t="n">
+        <v>-1.714502871247518</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>5</v>
+      </c>
+      <c r="B51" t="n">
+        <v>-1.714502871054043</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>1</v>
+      </c>
+      <c r="B52" t="n">
+        <v>0.08478485128744218</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" t="n">
+        <v>0.08478485149723949</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>3</v>
+      </c>
+      <c r="B54" t="n">
+        <v>-0.008533291523682623</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>4</v>
+      </c>
+      <c r="B55" t="n">
+        <v>0.004929485612566453</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>5</v>
+      </c>
+      <c r="B56" t="n">
+        <v>0.01228372537992581</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>1</v>
+      </c>
+      <c r="B57" t="n">
+        <v>-1.301030758081586</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>2</v>
+      </c>
+      <c r="B58" t="n">
+        <v>-1.106809010865079</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>3</v>
+      </c>
+      <c r="B59" t="n">
+        <v>-1.000204972662648</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>4</v>
+      </c>
+      <c r="B60" t="n">
+        <v>-0.9792985372673635</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B61" t="n">
+        <v>-0.8967147707367943</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>1</v>
+      </c>
+      <c r="B62" t="n">
+        <v>0.441967577125172</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>2</v>
+      </c>
+      <c r="B63" t="n">
+        <v>0.4341749805396881</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>3</v>
+      </c>
+      <c r="B64" t="n">
+        <v>0.4429988947823184</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>4</v>
+      </c>
+      <c r="B65" t="n">
+        <v>0.4632403319527937</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>5</v>
+      </c>
+      <c r="B66" t="n">
+        <v>0.4692072429771941</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>1</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0.3953639339562841</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>2</v>
+      </c>
+      <c r="B68" t="n">
+        <v>0.3856014510772848</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>3</v>
+      </c>
+      <c r="B69" t="n">
+        <v>0.4367893717032261</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>4</v>
+      </c>
+      <c r="B70" t="n">
+        <v>0.4419980120622632</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>5</v>
+      </c>
+      <c r="B71" t="n">
+        <v>0.3970253368711549</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>1</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-0.04470876910751945</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>2</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-0.04470876910679204</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>3</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-0.04470876910750354</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>4</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-0.04470876910750402</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>5</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-0.04470876910749758</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>1</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-1.084638193602981</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>2</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-1.084635875904093</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>3</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-1.084635875903832</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>4</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-1.084596930475571</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>5</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-1.084596816955205</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>1</v>
+      </c>
+      <c r="B82" t="n">
+        <v>0.04579747052962768</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>2</v>
+      </c>
+      <c r="B83" t="n">
+        <v>0.04579747051893731</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>3</v>
+      </c>
+      <c r="B84" t="n">
+        <v>0.04579746351818592</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>4</v>
+      </c>
+      <c r="B85" t="n">
+        <v>0.04579745442420143</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>5</v>
+      </c>
+      <c r="B86" t="n">
         <v>0.04579747050928459</v>
       </c>
     </row>

</xml_diff>